<commit_message>
feat: fix template download reliability and update static template with subject column
</commit_message>
<xml_diff>
--- a/backend/templates/question_import_template.xlsx
+++ b/backend/templates/question_import_template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="题库模板" sheetId="1" r:id="rId1"/>
+    <sheet name="题目导入模板" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,16 +407,16 @@
         <v>题干</v>
       </c>
       <c r="C1" t="str">
-        <v>选项A</v>
+        <v>A选项</v>
       </c>
       <c r="D1" t="str">
-        <v>选项B</v>
+        <v>B选项</v>
       </c>
       <c r="E1" t="str">
-        <v>选项C</v>
+        <v>C选项</v>
       </c>
       <c r="F1" t="str">
-        <v>选项D</v>
+        <v>D选项</v>
       </c>
       <c r="G1" t="str">
         <v>答案</v>
@@ -435,14 +435,17 @@
       </c>
       <c r="L1" t="str">
         <v>状态</v>
+      </c>
+      <c r="M1" t="str">
+        <v>学科</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>single</v>
+        <v>单选</v>
       </c>
       <c r="B2" t="str">
-        <v>以下哪项是JavaScript运行时？</v>
+        <v>下列哪一个是 JavaScript 运行时环境？</v>
       </c>
       <c r="C2" t="str">
         <v>Node.js</v>
@@ -460,24 +463,27 @@
         <v>A</v>
       </c>
       <c r="H2" t="str">
-        <v>Node.js 是 JavaScript 运行时。</v>
+        <v>Node.js 是 JavaScript 运行时环境。</v>
       </c>
       <c r="I2" t="str">
         <v>编程基础,JavaScript</v>
       </c>
-      <c r="J2">
+      <c r="J2" t="str">
         <v>2</v>
       </c>
       <c r="K2" t="str">
-        <v>第一章</v>
+        <v>第1章</v>
       </c>
       <c r="L2" t="str">
         <v>published</v>
+      </c>
+      <c r="M2" t="str">
+        <v>英语</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>